<commit_message>
Add delivery brief page mapping each deliverable requirement
- docs/brief.html: deliverables checklist, three-layer model and flow,
  automatic vs human-judgement table with sample examples, matching basis
  and risk controls, provenance, maintenance, sample results, demo route.
- Link it from every page, the index and the README.
- Regenerate docs/samples with the current code; fix auto-merge count
  for the supplier C PDF in the design doc (5, not 6).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XaZ8tHW45oZH5BjVy672tV
</commit_message>
<xml_diff>
--- a/docs/samples/import_report.xlsx
+++ b/docs/samples/import_report.xlsx
@@ -562,7 +562,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-23 06:28</t>
+          <t>2026-09-23 08:30</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -625,7 +625,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-23 06:28</t>
+          <t>2026-09-23 08:30</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -688,7 +688,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-23 06:28</t>
+          <t>2026-09-23 08:30</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -751,7 +751,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-23 06:28</t>
+          <t>2026-09-23 08:30</t>
         </is>
       </c>
       <c r="F5" t="n">

</xml_diff>

<commit_message>
Update docs and samples for the review-driven rule changes
- Design doc: import failure and retry, web preview, normalized identity,
  latest-value stance on key-attribute changes, data-quality checks,
  soft package size, year-overlap handling, grouped review, revision log.
- Delivery brief: auto vs human tables, why the 12 auto-merges are safe
  and how to switch them off, updated entry points, numbers and demo route.
- PRD and implementation doc aligned; samples regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XaZ8tHW45oZH5BjVy672tV
</commit_message>
<xml_diff>
--- a/docs/samples/import_report.xlsx
+++ b/docs/samples/import_report.xlsx
@@ -562,7 +562,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-23 08:30</t>
+          <t>2026-09-23 14:12</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -595,7 +595,7 @@
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026.09-1</t>
+          <t>2026.09-2</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-23 08:30</t>
+          <t>2026-09-23 14:12</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -658,7 +658,7 @@
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026.09-1</t>
+          <t>2026.09-2</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-23 08:30</t>
+          <t>2026-09-23 14:12</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -721,7 +721,7 @@
       <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026.09-1</t>
+          <t>2026.09-2</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-23 08:30</t>
+          <t>2026-09-23 14:12</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -784,7 +784,7 @@
       <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026.09-1</t>
+          <t>2026.09-2</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr">
@@ -1990,7 +1990,7 @@
       <c r="E50" t="inlineStr"/>
       <c r="F50" t="inlineStr">
         <is>
-          <t>MISSING_CURRENCY, MISSING_OE, MISSING_PRICE</t>
+          <t>MISSING_CURRENCY, MISSING_OE, MISSING_PRICE, SUSPECTED_NAME_ERROR</t>
         </is>
       </c>
     </row>
@@ -2066,7 +2066,11 @@
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr"/>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>SUSPECTED_NAME_ERROR</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">

</xml_diff>

<commit_message>
Update docs and samples for re-normalization and import diff changes
- Design: unchanged = same raw row and mapping, package size change is an
  update, run_matching re-normalizes before matching, revision log.
- Brief, PRD and implementation doc: new A v2 results, rule-change demo
  step (add a synonym, run run_matching), --noinput on every demo command.
- Samples regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XaZ8tHW45oZH5BjVy672tV
</commit_message>
<xml_diff>
--- a/docs/samples/import_report.xlsx
+++ b/docs/samples/import_report.xlsx
@@ -562,7 +562,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-23 14:12</t>
+          <t>2026-09-23 23:50</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -625,7 +625,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-23 14:12</t>
+          <t>2026-09-23 23:50</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -688,7 +688,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-23 14:12</t>
+          <t>2026-09-23 23:50</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -698,13 +698,13 @@
         <v>3</v>
       </c>
       <c r="H4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="I4" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K4" t="n">
         <v>0</v>
@@ -726,7 +726,7 @@
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>4601cb5d75e62532</t>
+          <t>05bb36358d92c7fc</t>
         </is>
       </c>
     </row>
@@ -751,7 +751,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-23 14:12</t>
+          <t>2026-09-23 23:50</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -2220,17 +2220,13 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>冲突</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>关键属性变化：dims: [151.0, 91.0, 14.0] → [151.0, 91.0, 20.0]</t>
-        </is>
-      </c>
+          <t>更新</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr">
         <is>
-          <t>KEY_ATTR_CHANGED</t>
+          <t>PACKAGE_DIMS_CHANGED</t>
         </is>
       </c>
     </row>
@@ -2360,11 +2356,19 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>未变</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr"/>
-      <c r="F66" t="inlineStr"/>
+          <t>冲突</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>关键属性变化：fitment: Volvo VN 2004-2017 → Volvo VN 2006-2017</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>KEY_ATTR_CHANGED</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">

</xml_diff>

<commit_message>
Document search-then-export and add a search export sample
- Design 6.1 (query and export) and a trade-off row; PRD F4 acceptance;
  brief deliverables and demo route; implementation doc; index and README.
- docs/samples/search_result_OE-VNL-1001.xlsx; other samples regenerated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XaZ8tHW45oZH5BjVy672tV
</commit_message>
<xml_diff>
--- a/docs/samples/import_report.xlsx
+++ b/docs/samples/import_report.xlsx
@@ -562,7 +562,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-23 23:50</t>
+          <t>2026-09-24 00:41</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -625,7 +625,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-23 23:50</t>
+          <t>2026-09-24 00:41</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -688,7 +688,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-23 23:50</t>
+          <t>2026-09-24 00:41</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -751,7 +751,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-23 23:50</t>
+          <t>2026-09-24 00:41</t>
         </is>
       </c>
       <c r="F5" t="n">

</xml_diff>

<commit_message>
Docs: check deliverables against the brief; refresh samples
- Delivery brief: demo steps create a login account (all pages need login)
  and mention publishing via Cloudflare Tunnel; extensions row (images,
  stock, SKU table sorting); review groups show SKU images.
- PRD and design: SKU table sorting.
- Samples regenerated with the current export format (stock sheet and
  columns).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XaZ8tHW45oZH5BjVy672tV
</commit_message>
<xml_diff>
--- a/docs/samples/import_report.xlsx
+++ b/docs/samples/import_report.xlsx
@@ -562,7 +562,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-09-24 00:41</t>
+          <t>2026-09-28 16:40</t>
         </is>
       </c>
       <c r="F2" t="n">
@@ -625,7 +625,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-09-24 00:41</t>
+          <t>2026-09-28 16:40</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -688,7 +688,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-09-24 00:41</t>
+          <t>2026-09-28 16:40</t>
         </is>
       </c>
       <c r="F4" t="n">
@@ -751,7 +751,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-09-24 00:41</t>
+          <t>2026-09-28 16:40</t>
         </is>
       </c>
       <c r="F5" t="n">

</xml_diff>